<commit_message>
fix: adjust weekly day counts for capacity report
Update first_w_days from 25 to 22 and second_w_days from 24 to 25 to correct the calculation of blank days in the capacity report template.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\1. Work\1. Daily\Capacity Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38BDFB9D-3AD6-4D0F-B8D9-A4AF144AED36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08585676-006E-4F97-9BE7-218C847D9F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-120" windowWidth="19800" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -688,7 +688,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -757,11 +757,7 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="7" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -782,6 +778,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1103,18 +1101,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="57" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
+      <c r="A1" s="53" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
       <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1142,24 +1140,24 @@
       <c r="R2" s="17"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="C3" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="62" t="s">
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="58" t="s">
         <v>119</v>
       </c>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="57"/>
       <c r="K3" s="5"/>
       <c r="L3" s="18" t="s">
         <v>5</v>
@@ -1184,15 +1182,15 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="64"/>
-      <c r="B4" s="64"/>
+      <c r="A4" s="60"/>
+      <c r="B4" s="60"/>
       <c r="C4" s="50">
         <f ca="1">TODAY()</f>
-        <v>46113</v>
+        <v>46117</v>
       </c>
       <c r="D4" s="50">
         <f ca="1">C4-1</f>
-        <v>46112</v>
+        <v>46116</v>
       </c>
       <c r="E4" s="51" t="s">
         <v>12</v>
@@ -1202,11 +1200,11 @@
       </c>
       <c r="G4" s="50">
         <f ca="1">TODAY()</f>
-        <v>46113</v>
+        <v>46117</v>
       </c>
       <c r="H4" s="50">
         <f ca="1">G4-1</f>
-        <v>46112</v>
+        <v>46116</v>
       </c>
       <c r="I4" s="51" t="s">
         <v>12</v>
@@ -1236,31 +1234,31 @@
       <c r="B5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="53">
-        <v>-513</v>
-      </c>
-      <c r="D5" s="53">
-        <v>-1062</v>
-      </c>
-      <c r="E5" s="53">
-        <v>-549</v>
-      </c>
-      <c r="F5" s="10">
+      <c r="C5" s="63">
+        <v>77</v>
+      </c>
+      <c r="D5" s="63">
+        <v>221</v>
+      </c>
+      <c r="E5" s="63">
+        <v>144</v>
+      </c>
+      <c r="F5" s="7">
         <f>C5/C60</f>
-        <v>-0.34803256445047492</v>
-      </c>
-      <c r="G5" s="54">
-        <v>622</v>
-      </c>
-      <c r="H5" s="54">
-        <v>739</v>
-      </c>
-      <c r="I5" s="54">
-        <v>117</v>
+        <v>5.2238805970149252E-2</v>
+      </c>
+      <c r="G5" s="63">
+        <v>1624</v>
+      </c>
+      <c r="H5" s="63">
+        <v>1627</v>
+      </c>
+      <c r="I5" s="63">
+        <v>3</v>
       </c>
       <c r="J5" s="7">
         <f t="shared" ref="J5:J12" si="0">G5/D60</f>
-        <v>0.37134328358208957</v>
+        <v>0.96955223880597019</v>
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="19" t="s">
@@ -1286,31 +1284,31 @@
       <c r="B6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="53">
-        <v>-32</v>
-      </c>
-      <c r="D6" s="53">
-        <v>-64</v>
-      </c>
-      <c r="E6" s="53">
-        <v>-32</v>
+      <c r="C6" s="52">
+        <v>-141</v>
+      </c>
+      <c r="D6" s="52">
+        <v>-128</v>
+      </c>
+      <c r="E6" s="63">
+        <v>13</v>
       </c>
       <c r="F6" s="10">
         <f t="shared" ref="F6:F11" si="1">C6/C61</f>
-        <v>-4.784688995215311E-2</v>
-      </c>
-      <c r="G6" s="53">
-        <v>-128</v>
-      </c>
-      <c r="H6" s="53">
-        <v>-134</v>
-      </c>
-      <c r="I6" s="53">
-        <v>-6</v>
-      </c>
-      <c r="J6" s="10">
+        <v>-0.21082535885167467</v>
+      </c>
+      <c r="G6" s="63">
+        <v>470</v>
+      </c>
+      <c r="H6" s="63">
+        <v>469</v>
+      </c>
+      <c r="I6" s="52">
+        <v>-1</v>
+      </c>
+      <c r="J6" s="7">
         <f t="shared" si="0"/>
-        <v>-0.16842105263157894</v>
+        <v>0.61842105263157898</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="19" t="s">
@@ -1334,31 +1332,31 @@
       <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="53">
-        <v>-335</v>
-      </c>
-      <c r="D7" s="53">
-        <v>-267</v>
-      </c>
-      <c r="E7" s="54">
-        <v>68</v>
-      </c>
-      <c r="F7" s="10">
+      <c r="C7" s="63">
+        <v>781</v>
+      </c>
+      <c r="D7" s="63">
+        <v>998</v>
+      </c>
+      <c r="E7" s="63">
+        <v>217</v>
+      </c>
+      <c r="F7" s="7">
         <f t="shared" si="1"/>
-        <v>-0.20022712330404638</v>
-      </c>
-      <c r="G7" s="54">
-        <v>1056</v>
-      </c>
-      <c r="H7" s="54">
-        <v>1211</v>
-      </c>
-      <c r="I7" s="54">
-        <v>155</v>
+        <v>0.46679815910585143</v>
+      </c>
+      <c r="G7" s="63">
+        <v>1354</v>
+      </c>
+      <c r="H7" s="63">
+        <v>1467</v>
+      </c>
+      <c r="I7" s="63">
+        <v>113</v>
       </c>
       <c r="J7" s="7">
         <f t="shared" si="0"/>
-        <v>0.55542406311637083</v>
+        <v>0.71216305062458907</v>
       </c>
       <c r="K7" s="5"/>
       <c r="L7" s="18" t="s">
@@ -1384,31 +1382,31 @@
       <c r="B8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="53">
-        <v>-391</v>
-      </c>
-      <c r="D8" s="53">
-        <v>-389</v>
-      </c>
-      <c r="E8" s="54">
-        <v>2</v>
+      <c r="C8" s="52">
+        <v>-380</v>
+      </c>
+      <c r="D8" s="52">
+        <v>-536</v>
+      </c>
+      <c r="E8" s="52">
+        <v>-156</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="1"/>
-        <v>-0.28390938135347082</v>
-      </c>
-      <c r="G8" s="53">
-        <v>-634</v>
-      </c>
-      <c r="H8" s="53">
-        <v>-207</v>
-      </c>
-      <c r="I8" s="54">
-        <v>427</v>
+        <v>-0.27592216090618643</v>
+      </c>
+      <c r="G8" s="52">
+        <v>-72</v>
+      </c>
+      <c r="H8" s="52">
+        <v>-142</v>
+      </c>
+      <c r="I8" s="52">
+        <v>-70</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="0"/>
-        <v>-0.40511182108626198</v>
+        <v>-4.6006389776357827E-2</v>
       </c>
       <c r="K8" s="5"/>
       <c r="L8" s="19" t="s">
@@ -1434,31 +1432,31 @@
       <c r="B9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="53">
-        <v>-119</v>
-      </c>
-      <c r="D9" s="53">
-        <v>-196</v>
-      </c>
-      <c r="E9" s="53">
-        <v>-77</v>
-      </c>
-      <c r="F9" s="10">
+      <c r="C9" s="63">
+        <v>104</v>
+      </c>
+      <c r="D9" s="52">
+        <v>-23</v>
+      </c>
+      <c r="E9" s="52">
+        <v>-127</v>
+      </c>
+      <c r="F9" s="7">
         <f t="shared" si="1"/>
-        <v>-8.9406461307287757E-2</v>
-      </c>
-      <c r="G9" s="54">
-        <v>592</v>
-      </c>
-      <c r="H9" s="54">
-        <v>1071</v>
-      </c>
-      <c r="I9" s="54">
-        <v>479</v>
+        <v>7.8136739293764093E-2</v>
+      </c>
+      <c r="G9" s="63">
+        <v>1442</v>
+      </c>
+      <c r="H9" s="63">
+        <v>1422</v>
+      </c>
+      <c r="I9" s="52">
+        <v>-20</v>
       </c>
       <c r="J9" s="7">
         <f t="shared" si="0"/>
-        <v>0.39140495867768593</v>
+        <v>0.95338842975206617</v>
       </c>
       <c r="K9" s="5"/>
       <c r="L9" s="19" t="s">
@@ -1484,31 +1482,31 @@
       <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="53">
-        <v>-703</v>
-      </c>
-      <c r="D10" s="53">
-        <v>-217</v>
-      </c>
-      <c r="E10" s="54">
-        <v>486</v>
-      </c>
-      <c r="F10" s="10">
+      <c r="C10" s="63">
+        <v>883</v>
+      </c>
+      <c r="D10" s="63">
+        <v>936</v>
+      </c>
+      <c r="E10" s="63">
+        <v>53</v>
+      </c>
+      <c r="F10" s="7">
         <f t="shared" si="1"/>
-        <v>-0.2958754208754209</v>
-      </c>
-      <c r="G10" s="54">
-        <v>1569</v>
-      </c>
-      <c r="H10" s="54">
-        <v>1732</v>
-      </c>
-      <c r="I10" s="54">
-        <v>163</v>
+        <v>0.37163299663299665</v>
+      </c>
+      <c r="G10" s="63">
+        <v>2288</v>
+      </c>
+      <c r="H10" s="63">
+        <v>2287</v>
+      </c>
+      <c r="I10" s="52">
+        <v>-1</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="0"/>
-        <v>0.58111111111111113</v>
+        <v>0.84740740740740739</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="19" t="s">
@@ -1532,31 +1530,31 @@
       <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="54">
-        <v>322</v>
-      </c>
-      <c r="D11" s="54">
-        <v>288</v>
-      </c>
-      <c r="E11" s="53">
-        <v>-34</v>
+      <c r="C11" s="63">
+        <v>356</v>
+      </c>
+      <c r="D11" s="63">
+        <v>426</v>
+      </c>
+      <c r="E11" s="63">
+        <v>70</v>
       </c>
       <c r="F11" s="7">
         <f t="shared" si="1"/>
-        <v>0.36960514233241504</v>
-      </c>
-      <c r="G11" s="54">
-        <v>628</v>
-      </c>
-      <c r="H11" s="54">
-        <v>772</v>
-      </c>
-      <c r="I11" s="54">
-        <v>144</v>
+        <v>0.40863177226813591</v>
+      </c>
+      <c r="G11" s="63">
+        <v>988</v>
+      </c>
+      <c r="H11" s="63">
+        <v>988</v>
+      </c>
+      <c r="I11" s="63">
+        <v>0</v>
       </c>
       <c r="J11" s="7">
         <f t="shared" si="0"/>
-        <v>0.63434343434343432</v>
+        <v>0.99797979797979797</v>
       </c>
       <c r="K11" s="5"/>
       <c r="L11" s="18" t="s">
@@ -1582,31 +1580,31 @@
       <c r="B12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="55">
-        <v>-1769</v>
-      </c>
-      <c r="D12" s="55">
-        <v>-1908</v>
-      </c>
-      <c r="E12" s="55">
-        <v>-139</v>
-      </c>
-      <c r="F12" s="52">
+      <c r="C12" s="64">
+        <v>1680</v>
+      </c>
+      <c r="D12" s="64">
+        <v>1895</v>
+      </c>
+      <c r="E12" s="64">
+        <v>215</v>
+      </c>
+      <c r="F12" s="9">
         <f>C12/C67</f>
-        <v>-0.18132617185498007</v>
-      </c>
-      <c r="G12" s="56">
-        <v>3707</v>
-      </c>
-      <c r="H12" s="56">
-        <v>5184</v>
-      </c>
-      <c r="I12" s="56">
-        <v>1477</v>
+        <v>0.17193208682570385</v>
+      </c>
+      <c r="G12" s="64">
+        <v>8094</v>
+      </c>
+      <c r="H12" s="64">
+        <v>8118</v>
+      </c>
+      <c r="I12" s="64">
+        <v>24</v>
       </c>
       <c r="J12" s="9">
         <f t="shared" si="0"/>
-        <v>0.33437817115796598</v>
+        <v>0.72894292468760558</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="19" t="s">
@@ -1632,24 +1630,24 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="65"/>
-      <c r="B13" s="61"/>
-      <c r="C13" s="66" t="s">
+      <c r="A13" s="61"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="61"/>
-      <c r="E13" s="66">
+      <c r="D13" s="57"/>
+      <c r="E13" s="62">
         <v>22</v>
       </c>
-      <c r="F13" s="61"/>
-      <c r="G13" s="66" t="s">
+      <c r="F13" s="57"/>
+      <c r="G13" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="61"/>
-      <c r="I13" s="66">
+      <c r="H13" s="57"/>
+      <c r="I13" s="62">
         <v>25</v>
       </c>
-      <c r="J13" s="61"/>
+      <c r="J13" s="57"/>
       <c r="K13" s="5"/>
       <c r="L13" s="19" t="s">
         <v>19</v>
@@ -3320,15 +3318,15 @@
         <v>98</v>
       </c>
       <c r="B67" s="5">
-        <v>8869</v>
+        <v>8883</v>
       </c>
       <c r="C67" s="5">
         <f t="shared" si="3"/>
-        <v>9755.9</v>
+        <v>9771.2999999999993</v>
       </c>
       <c r="D67" s="5">
         <f t="shared" si="2"/>
-        <v>11086.25</v>
+        <v>11103.75</v>
       </c>
       <c r="L67" s="27"/>
       <c r="M67" s="27"/>

</xml_diff>